<commit_message>
Reuse detail image for third carousel slot in trial
</commit_message>
<xml_diff>
--- a/temu-trial/SKU-image-report.xlsx
+++ b/temu-trial/SKU-image-report.xlsx
@@ -555,7 +555,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>产地、价格、材料、食品接触材质、圆形规格、包装尺寸及重量已补充；仅2张原图，不足3张；库存引用10.9表格，未验证实时库存；尚未测试TEMU导入</t>
+          <t>已按用户要求将详情图复用为第3个轮播图；3个轮播图位置均已填入，但第1与第3张为同图，共2张不同原图。尚未验证TEMU是否接受重复图或国内网络访问。库存为10.9表格快照。</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -9059,7 +9059,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A8"/>
+  <dimension ref="A1:A9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="56" customWidth="1" min="1" max="1"/>
@@ -9117,7 +9117,14 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>样本仍缺第3张有效轮播原图；未执行TEMU上传，未验证中国大陆网络图片访问。</t>
+          <t>按用户要求将详情图URL复用至第3个轮播图位置，第1与第3张重复；尚未验证TEMU是否接受重复图及中国大陆访问。未上传TEMU。</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>轮播图与详情图允许共用（用户确认）；本次将BY6的图片URL填写到BQ6。</t>
         </is>
       </c>
     </row>

</xml_diff>